<commit_message>
Endpoints Compeleted & Pagination Added
</commit_message>
<xml_diff>
--- a/backend/docs/Backend-Proje-Plani-Takip.xlsx
+++ b/backend/docs/Backend-Proje-Plani-Takip.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mehmet\Desktop\personal-blog\backend\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D1F687-F218-41DD-80F9-BF44BF23D843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{435CA61F-4410-4F73-B8AF-1E6BC4A4B636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,15 +34,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="267">
   <si>
     <t>Faz</t>
   </si>
@@ -92,12 +89,18 @@
     <t>B-03</t>
   </si>
   <si>
+    <t>✓</t>
+  </si>
+  <si>
     <t>0.2</t>
   </si>
   <si>
     <t>git rm -r --cached myvenv dev.db v1_db.db ile takipten çıkar ve commit'le</t>
   </si>
   <si>
+    <t>Kontrol edilemedi: git deposu bu klasörde görünmüyor. 'git ls-files myvenv dev.db v1_db.db' boş dönmeli.</t>
+  </si>
+  <si>
     <t>0.3</t>
   </si>
   <si>
@@ -107,6 +110,9 @@
     <t>B-02</t>
   </si>
   <si>
+    <t>requirements.txt düzgün ve pinli. Eksik: requirements-dev.txt henüz yok (test bağımlılıkları gelince ayır).</t>
+  </si>
+  <si>
     <t>0.4</t>
   </si>
   <si>
@@ -191,6 +197,9 @@
     <t>B-05</t>
   </si>
   <si>
+    <t>⚠ Kısmen: GET route'ları ProjectRead dönüyor; POST, PATCH ve PUT /slug route'larında response_model yok → tablo modeli (snake_case) dönüyor.</t>
+  </si>
+  <si>
     <t>1.4</t>
   </si>
   <si>
@@ -221,6 +230,9 @@
     <t>B-07, B-09</t>
   </si>
   <si>
+    <t>⚠ Kısmen: PATCH exclude_unset ile çalışıyor. get_by_slug ise hâlâ BaseRepository içinde (ProjectRepository'de override edilmiş).</t>
+  </si>
+  <si>
     <t>1.7</t>
   </si>
   <si>
@@ -230,6 +242,9 @@
     <t>B-07, B-21</t>
   </si>
   <si>
+    <t>Kısmen: PUT/PATCH/DELETE route'ları var. Page[T] sayfalama şeması yok (get_all düz liste dönüyor).</t>
+  </si>
+  <si>
     <t>1.8</t>
   </si>
   <si>
@@ -239,12 +254,18 @@
     <t>B-08</t>
   </si>
   <si>
+    <t>Yapılmadı: db_dependency'de try/except/rollback yok.</t>
+  </si>
+  <si>
     <t>1.K</t>
   </si>
   <si>
     <t>KONTROL: /docs'ta 5 project endpoint'i; POST id istemiyor; PATCH tek alan güncelliyor</t>
   </si>
   <si>
+    <t>Doğrulandı: POST id istemiyor, PATCH tek alan güncelliyor, projects için PUT/PATCH/DELETE route'ları /docs'ta var.</t>
+  </si>
+  <si>
     <t>Faz 2 — Test Altyapısı</t>
   </si>
   <si>
@@ -260,6 +281,9 @@
     <t>B-14</t>
   </si>
   <si>
+    <t>Yapılmadı: tests/ klasörü yok.</t>
+  </si>
+  <si>
     <t>2.2</t>
   </si>
   <si>
@@ -287,6 +311,9 @@
     <t>B-06</t>
   </si>
   <si>
+    <t>Yapılmadı: alembic/ klasörü yok; db.py hâlâ create_all kullanıyor.</t>
+  </si>
+  <si>
     <t>3.2</t>
   </si>
   <si>
@@ -371,12 +398,18 @@
     <t>24.08.2026 Pzt</t>
   </si>
   <si>
+    <t>Taslak var (models/user.py) ama table=True değil, hashed_password/is_active/is_admin yok.</t>
+  </si>
+  <si>
     <t>5.2</t>
   </si>
   <si>
     <t>core/security.py: pwdlib[argon2] ile hash/verify + PyJWT ile access token üret/çöz</t>
   </si>
   <si>
+    <t>core/security.py şu an boş (0 bayt).</t>
+  </si>
+  <si>
     <t>5.3</t>
   </si>
   <si>
@@ -425,6 +458,9 @@
     <t>Faz 5</t>
   </si>
   <si>
+    <t>Kısmen: imagekitio==5.9.0 pinli. IMAGEKIT_* ayarları Settings'te yok.</t>
+  </si>
+  <si>
     <t>6.2</t>
   </si>
   <si>
@@ -482,6 +518,9 @@
     <t>B-22</t>
   </si>
   <si>
+    <t>Yapılmadı: Dockerfile yok.</t>
+  </si>
+  <si>
     <t>7.2</t>
   </si>
   <si>
@@ -801,9 +840,6 @@
   </si>
   <si>
     <t>Yerel Python 3.14 çok yeni; Docker imajında 3.12 gibi oturmuş sürüm tercih edilmeli</t>
-  </si>
-  <si>
-    <t>✓</t>
   </si>
 </sst>
 </file>
@@ -1332,7 +1368,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1358,19 +1394,19 @@
         <v>15</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J2" s="4"/>
     </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
@@ -1388,19 +1424,21 @@
         <v>15</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="J3" s="4"/>
-    </row>
-    <row r="4" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
@@ -1415,22 +1453,24 @@
         <v>14</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="J4" s="4"/>
-    </row>
-    <row r="5" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
@@ -1442,25 +1482,25 @@
         <v>0.75</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J5" s="4"/>
     </row>
-    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
@@ -1472,25 +1512,25 @@
         <v>0.33</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
@@ -1505,22 +1545,22 @@
         <v>14</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D8" s="3">
         <v>1</v>
@@ -1535,22 +1575,22 @@
         <v>14</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J8" s="4"/>
     </row>
-    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D9" s="3">
         <v>1</v>
@@ -1568,19 +1608,19 @@
         <v>14</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J9" s="4"/>
     </row>
-    <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D10" s="3">
         <v>1</v>
@@ -1592,239 +1632,247 @@
         <v>0.25</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>14</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D11" s="3">
         <v>2</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F11" s="6">
         <v>0.75</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D12" s="3">
         <v>2</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F12" s="6">
         <v>1.5</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D13" s="3">
         <v>2</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F13" s="6">
         <v>0.5</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="J13" s="4"/>
-    </row>
-    <row r="14" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D14" s="3">
         <v>2</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F14" s="6">
         <v>1.5</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J14" s="4"/>
     </row>
-    <row r="15" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D15" s="3">
         <v>3</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F15" s="6">
         <v>0.75</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>253</v>
+        <v>16</v>
       </c>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D16" s="3">
         <v>3</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F16" s="6">
         <v>1</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="J16" s="4"/>
-    </row>
-    <row r="17" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D17" s="3">
         <v>3</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F17" s="6">
         <v>1.5</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="I17" s="7"/>
-      <c r="J17" s="4"/>
-    </row>
-    <row r="18" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D18" s="3">
         <v>3</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F18" s="6">
         <v>0.33</v>
@@ -1833,116 +1881,126 @@
         <v>14</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="I18" s="7"/>
-      <c r="J18" s="4"/>
-    </row>
-    <row r="19" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="D19" s="3">
         <v>3</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F19" s="6">
         <v>0.25</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="I19" s="7"/>
-      <c r="J19" s="4"/>
-    </row>
-    <row r="20" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="I19" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="D20" s="3">
         <v>3</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F20" s="6">
         <v>2</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="I20" s="7"/>
-      <c r="J20" s="4"/>
-    </row>
-    <row r="21" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J20" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="D21" s="3">
         <v>3</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F21" s="6">
         <v>2</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="I21" s="7"/>
       <c r="J21" s="4"/>
     </row>
-    <row r="22" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="D22" s="3">
         <v>3</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F22" s="6">
         <v>0.25</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>14</v>
@@ -1950,83 +2008,85 @@
       <c r="I22" s="7"/>
       <c r="J22" s="4"/>
     </row>
-    <row r="23" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="D23" s="3">
         <v>4</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F23" s="6">
         <v>1.5</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I23" s="7"/>
-      <c r="J23" s="4"/>
-    </row>
-    <row r="24" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J23" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="D24" s="3">
         <v>4</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F24" s="6">
         <v>1</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I24" s="7"/>
       <c r="J24" s="4"/>
     </row>
-    <row r="25" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="D25" s="3">
         <v>4</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F25" s="6">
         <v>1.5</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>14</v>
@@ -2034,27 +2094,27 @@
       <c r="I25" s="7"/>
       <c r="J25" s="4"/>
     </row>
-    <row r="26" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D26" s="3">
         <v>4</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F26" s="6">
         <v>1</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>14</v>
@@ -2062,27 +2122,27 @@
       <c r="I26" s="7"/>
       <c r="J26" s="4"/>
     </row>
-    <row r="27" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="D27" s="3">
         <v>4</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F27" s="6">
         <v>0.25</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>14</v>
@@ -2090,27 +2150,27 @@
       <c r="I27" s="7"/>
       <c r="J27" s="4"/>
     </row>
-    <row r="28" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="D28" s="3">
         <v>5</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="F28" s="6">
         <v>2</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>14</v>
@@ -2118,27 +2178,27 @@
       <c r="I28" s="7"/>
       <c r="J28" s="4"/>
     </row>
-    <row r="29" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="D29" s="3">
         <v>5</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="F29" s="6">
         <v>1.5</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>14</v>
@@ -2146,27 +2206,27 @@
       <c r="I29" s="7"/>
       <c r="J29" s="4"/>
     </row>
-    <row r="30" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="D30" s="3">
         <v>5</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="F30" s="6">
         <v>1.5</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="H30" s="5" t="s">
         <v>14</v>
@@ -2174,27 +2234,27 @@
       <c r="I30" s="7"/>
       <c r="J30" s="4"/>
     </row>
-    <row r="31" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="D31" s="3">
         <v>6</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F31" s="6">
         <v>2</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="H31" s="5" t="s">
         <v>14</v>
@@ -2202,27 +2262,27 @@
       <c r="I31" s="7"/>
       <c r="J31" s="4"/>
     </row>
-    <row r="32" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="D32" s="3">
         <v>6</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F32" s="6">
         <v>1</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="H32" s="5" t="s">
         <v>14</v>
@@ -2230,27 +2290,27 @@
       <c r="I32" s="7"/>
       <c r="J32" s="4"/>
     </row>
-    <row r="33" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="D33" s="3">
         <v>6</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F33" s="6">
         <v>0.25</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H33" s="5" t="s">
         <v>14</v>
@@ -2258,251 +2318,257 @@
       <c r="I33" s="7"/>
       <c r="J33" s="4"/>
     </row>
-    <row r="34" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="D34" s="3">
         <v>7</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="F34" s="6">
         <v>1</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I34" s="7"/>
-      <c r="J34" s="4"/>
-    </row>
-    <row r="35" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J34" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="D35" s="3">
         <v>7</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="F35" s="6">
         <v>2</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I35" s="7"/>
-      <c r="J35" s="4"/>
-    </row>
-    <row r="36" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J35" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="D36" s="3">
         <v>7</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="F36" s="6">
         <v>1.5</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I36" s="7"/>
       <c r="J36" s="4"/>
     </row>
-    <row r="37" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="D37" s="3">
         <v>8</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="F37" s="6">
         <v>1.5</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I37" s="7"/>
       <c r="J37" s="4"/>
     </row>
-    <row r="38" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="D38" s="3">
         <v>8</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="F38" s="6">
         <v>1</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I38" s="7"/>
       <c r="J38" s="4"/>
     </row>
-    <row r="39" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="D39" s="3">
         <v>8</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="F39" s="6">
         <v>0.5</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="I39" s="7"/>
       <c r="J39" s="4"/>
     </row>
-    <row r="40" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="D40" s="3">
         <v>8</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="F40" s="6">
         <v>1</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="I40" s="7"/>
       <c r="J40" s="4"/>
     </row>
-    <row r="41" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="D41" s="3">
         <v>9</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="F41" s="6">
         <v>0.5</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="H41" s="5" t="s">
         <v>14</v>
       </c>
       <c r="I41" s="7"/>
-      <c r="J41" s="4"/>
-    </row>
-    <row r="42" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="J41" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="D42" s="3">
         <v>9</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="F42" s="6">
         <v>2.5</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="H42" s="5" t="s">
         <v>14</v>
@@ -2510,27 +2576,27 @@
       <c r="I42" s="7"/>
       <c r="J42" s="4"/>
     </row>
-    <row r="43" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="D43" s="3">
         <v>9</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="F43" s="6">
         <v>1.5</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="H43" s="5" t="s">
         <v>14</v>
@@ -2538,27 +2604,27 @@
       <c r="I43" s="7"/>
       <c r="J43" s="4"/>
     </row>
-    <row r="44" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="D44" s="3">
         <v>10</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="F44" s="6">
         <v>0.75</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="H44" s="5" t="s">
         <v>14</v>
@@ -2566,27 +2632,27 @@
       <c r="I44" s="7"/>
       <c r="J44" s="4"/>
     </row>
-    <row r="45" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="D45" s="3">
         <v>10</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="F45" s="6">
         <v>1.5</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="H45" s="5" t="s">
         <v>14</v>
@@ -2594,27 +2660,27 @@
       <c r="I45" s="7"/>
       <c r="J45" s="4"/>
     </row>
-    <row r="46" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="D46" s="3">
         <v>10</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="F46" s="6">
         <v>1.5</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H46" s="5" t="s">
         <v>14</v>
@@ -2622,27 +2688,27 @@
       <c r="I46" s="7"/>
       <c r="J46" s="4"/>
     </row>
-    <row r="47" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="D47" s="3">
         <v>10</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="F47" s="6">
         <v>0.5</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="H47" s="5" t="s">
         <v>14</v>
@@ -2650,55 +2716,57 @@
       <c r="I47" s="7"/>
       <c r="J47" s="4"/>
     </row>
-    <row r="48" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="D48" s="3">
         <v>11</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="F48" s="6">
         <v>2</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="I48" s="7"/>
-      <c r="J48" s="4"/>
-    </row>
-    <row r="49" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J48" s="4" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="D49" s="3">
         <v>11</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="F49" s="6">
         <v>2</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="H49" s="5" t="s">
         <v>14</v>
@@ -2706,27 +2774,27 @@
       <c r="I49" s="7"/>
       <c r="J49" s="4"/>
     </row>
-    <row r="50" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="D50" s="3">
         <v>11</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="F50" s="6">
         <v>1</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="H50" s="5" t="s">
         <v>14</v>
@@ -2734,21 +2802,21 @@
       <c r="I50" s="7"/>
       <c r="J50" s="4"/>
     </row>
-    <row r="51" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="D51" s="3">
         <v>12</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="F51" s="6">
         <v>1.5</v>
@@ -2757,26 +2825,26 @@
         <v>14</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="I51" s="7"/>
       <c r="J51" s="4"/>
     </row>
-    <row r="52" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="D52" s="3">
         <v>12</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="F52" s="6">
         <v>1.5</v>
@@ -2790,27 +2858,27 @@
       <c r="I52" s="7"/>
       <c r="J52" s="4"/>
     </row>
-    <row r="53" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="D53" s="3">
         <v>12</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="F53" s="6">
         <v>1</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="H53" s="5" t="s">
         <v>14</v>
@@ -2818,55 +2886,55 @@
       <c r="I53" s="7"/>
       <c r="J53" s="4"/>
     </row>
-    <row r="54" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="D54" s="3">
         <v>13</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="F54" s="6">
         <v>0.5</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I54" s="7"/>
       <c r="J54" s="4"/>
     </row>
-    <row r="55" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="D55" s="3">
         <v>13</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="F55" s="6">
         <v>1</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="H55" s="5" t="s">
         <v>14</v>
@@ -2874,27 +2942,27 @@
       <c r="I55" s="7"/>
       <c r="J55" s="4"/>
     </row>
-    <row r="56" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="D56" s="3">
         <v>13</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="F56" s="6">
         <v>0.25</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="H56" s="5" t="s">
         <v>14</v>
@@ -2902,27 +2970,27 @@
       <c r="I56" s="7"/>
       <c r="J56" s="4"/>
     </row>
-    <row r="57" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="D57" s="3">
         <v>14</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="F57" s="6">
         <v>1.5</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="H57" s="5" t="s">
         <v>14</v>
@@ -2930,27 +2998,27 @@
       <c r="I57" s="7"/>
       <c r="J57" s="4"/>
     </row>
-    <row r="58" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="D58" s="3">
         <v>14</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="F58" s="6">
         <v>1</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="H58" s="5" t="s">
         <v>14</v>
@@ -2958,27 +3026,27 @@
       <c r="I58" s="7"/>
       <c r="J58" s="4"/>
     </row>
-    <row r="59" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="D59" s="3">
         <v>14</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="F59" s="6">
         <v>1</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="H59" s="5" t="s">
         <v>14</v>
@@ -2986,27 +3054,27 @@
       <c r="I59" s="7"/>
       <c r="J59" s="4"/>
     </row>
-    <row r="60" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="D60" s="3">
         <v>14</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="F60" s="6">
         <v>0.5</v>
       </c>
       <c r="G60" s="5" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="H60" s="5" t="s">
         <v>14</v>
@@ -3043,19 +3111,19 @@
     <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3066,16 +3134,16 @@
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -3105,7 +3173,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B7" s="12">
         <f>COUNTIF('Görev Takibi'!$A$2:$A$60,$A7)</f>
@@ -3113,7 +3181,7 @@
       </c>
       <c r="C7" s="12">
         <f>COUNTIFS('Görev Takibi'!$A$2:$A$60,$A7,'Görev Takibi'!$I$2:$I$60,"✓")</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D7" s="13">
         <f>SUMIF('Görev Takibi'!$A$2:$A$60,$A7,'Görev Takibi'!$F$2:$F$60)</f>
@@ -3121,16 +3189,16 @@
       </c>
       <c r="E7" s="13">
         <f>SUMIFS('Görev Takibi'!$F$2:$F$60,'Görev Takibi'!$A$2:$A$60,$A7,'Görev Takibi'!$I$2:$I$60,"✓")</f>
-        <v>6</v>
+        <v>8.08</v>
       </c>
       <c r="F7" s="14">
         <f t="shared" si="0"/>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B8" s="12">
         <f>COUNTIF('Görev Takibi'!$A$2:$A$60,$A8)</f>
@@ -3155,7 +3223,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B9" s="12">
         <f>COUNTIF('Görev Takibi'!$A$2:$A$60,$A9)</f>
@@ -3180,7 +3248,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B10" s="12">
         <f>COUNTIF('Görev Takibi'!$A$2:$A$60,$A10)</f>
@@ -3205,7 +3273,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B11" s="12">
         <f>COUNTIF('Görev Takibi'!$A$2:$A$60,$A11)</f>
@@ -3230,7 +3298,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="B12" s="12">
         <f>COUNTIF('Görev Takibi'!$A$2:$A$60,$A12)</f>
@@ -3255,7 +3323,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B13" s="12">
         <f>COUNTIF('Görev Takibi'!$A$2:$A$60,$A13)</f>
@@ -3280,7 +3348,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B14" s="12">
         <f>COUNTIF('Görev Takibi'!$A$2:$A$60,$A14)</f>
@@ -3305,7 +3373,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="B15" s="16">
         <f>SUM(B6:B14)</f>
@@ -3313,7 +3381,7 @@
       </c>
       <c r="C15" s="16">
         <f>SUM(C6:C14)</f>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D15" s="17">
         <f>SUM(D6:D14)</f>
@@ -3321,21 +3389,21 @@
       </c>
       <c r="E15" s="17">
         <f>SUM(E6:E14)</f>
-        <v>9.83</v>
+        <v>11.91</v>
       </c>
       <c r="F15" s="18">
         <f t="shared" si="0"/>
-        <v>0.25423728813559321</v>
+        <v>0.30508474576271188</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -3359,417 +3427,441 @@
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="F2" s="7"/>
     </row>
-    <row r="3" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>207</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="22" t="s">
-        <v>193</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="7"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F3" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="F4" s="7"/>
     </row>
-    <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="F5" s="7"/>
-    </row>
-    <row r="6" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="E6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
+        <v>230</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="21" t="s">
+        <v>234</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="21" t="s">
+        <v>237</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="21" t="s">
+        <v>239</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F6" s="7"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>203</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="F7" s="7"/>
-    </row>
-    <row r="8" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>203</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="F8" s="7"/>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
+      <c r="F13" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>254</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="25" t="s">
+        <v>254</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="21" t="s">
+        <v>258</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>254</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="21" t="s">
+        <v>261</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>254</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="21" t="s">
+        <v>264</v>
+      </c>
+      <c r="B22" s="25" t="s">
+        <v>254</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="23" t="s">
-        <v>203</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F9" s="7"/>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
-        <v>216</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="7"/>
-    </row>
-    <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="s">
-        <v>220</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" s="7"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" s="7"/>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
-        <v>225</v>
-      </c>
-      <c r="B13" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="F13" s="7"/>
-    </row>
-    <row r="14" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="B14" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="F14" s="7"/>
-    </row>
-    <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="B15" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="F15" s="7"/>
-    </row>
-    <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="F16" s="7"/>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="F17" s="7"/>
-    </row>
-    <row r="18" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="21" t="s">
-        <v>239</v>
-      </c>
-      <c r="B18" s="25" t="s">
-        <v>240</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F18" s="7"/>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="25" t="s">
-        <v>240</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F19" s="7"/>
-    </row>
-    <row r="20" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
-        <v>244</v>
-      </c>
-      <c r="B20" s="25" t="s">
-        <v>240</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F20" s="7"/>
-    </row>
-    <row r="21" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="21" t="s">
-        <v>247</v>
-      </c>
-      <c r="B21" s="25" t="s">
-        <v>240</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F21" s="7"/>
-    </row>
-    <row r="22" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="21" t="s">
-        <v>250</v>
-      </c>
-      <c r="B22" s="25" t="s">
-        <v>240</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="F22" s="7"/>
     </row>
-    <row r="23" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="F23" s="7"/>
     </row>

</xml_diff>

<commit_message>
Blog Module Completed & User Model Added
</commit_message>
<xml_diff>
--- a/backend/docs/Backend-Proje-Plani-Takip.xlsx
+++ b/backend/docs/Backend-Proje-Plani-Takip.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Görev Takibi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Özet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Denetim Bulguları" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Görev Takibi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Özet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Denetim Bulguları" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Görev Takibi'!$A$1:$J$60</definedName>
@@ -1766,7 +1766,7 @@
     <row r="28" ht="25.5" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Faz 4 — Blog (Post) Modülü</t>
+          <t>Faz 4 — Blog Modülü</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Post modeli: title, slug (unique+index), summary, content (Text), cover_image_url, tags, status, published_at, reading_time</t>
+          <t>Blog modeli (tablo: blogs): title, slug (unique+index), summary, content (Text), cover_img_url, tags (JSON), is_published, featured, reading_time</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1800,13 +1800,21 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I28" s="7" t="n"/>
-      <c r="J28" s="4" t="n"/>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: models/blog.py (tablo blogs). Kararlar: status yerine is_published + featured; yayın tarihi için created_at kullanılıyor (published_at yok); reading_time saklanan kolon, sunucu hesaplar (utils/reading_time.py). BaseModel: created_at/updated_at sa_type=DateTime(timezone=True), onupdate=utcnow (sa_column ortak taban sınıfta tabloya iki kez bağlanıyordu).</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Faz 4 — Blog (Post) Modülü</t>
+          <t>Faz 4 — Blog Modülü</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1816,7 +1824,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>PostCreate/Update/Read şemaları; python-slugify ile Türkçe karakter → ASCII slug</t>
+          <t>BlogCreate / BlogUpdate / BlogRead / BlogListItem şemaları; slug sunucuda üretilir (utils/slug.py), şemalarda yok</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1840,13 +1848,21 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I29" s="7" t="n"/>
-      <c r="J29" s="4" t="n"/>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: schemas/blog.py. reading_time yalnızca okuma şemalarında, slug şemalarda yok. BlogListItem içeriksiz liste şeması (Page[BlogListItem] için).</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="25.5" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Faz 4 — Blog (Post) Modülü</t>
+          <t>Faz 4 — Blog Modülü</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1856,7 +1872,7 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>PostRepository: slug ile getir, sadece published listele, tag filtresi, published_at DESC sırala</t>
+          <t>BlogRepository: slug ile getir, yalnızca yayınlanmış (is_published) listele, tag filtresi, created_at DESC sırala</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1880,13 +1896,21 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I30" s="7" t="n"/>
-      <c r="J30" s="4" t="n"/>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: repositories/blog.py. _before_save kancası (base put/patch) ile reading_time içerik değişince yeniden hesaplanır; get_by_id/get_by_slug published_only parametresi (varsayılan False, admin taslakları görür); get_published_page: is_published filtresi, created_at DESC, tag filtresi (JSON metninde tırnaklı LIKE). BlogListItem içeriksiz.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Faz 4 — Blog (Post) Modülü</t>
+          <t>Faz 4 — Blog Modülü</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1896,7 +1920,7 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>/api/v1/posts endpoint'leri: public list (published), public get-by-slug, admin CRUD</t>
+          <t>/api/v1/blogs endpoint'leri: public list (BlogListItem, yalnızca yayınlanmış), public get-by-slug, admin CRUD</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1920,13 +1944,21 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="4" t="n"/>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: public (api/v1/blogs.py: liste Page[BlogListItem] + tag filtresi, GET /{id}, GET /slug/{slug}; yayınlanmamış → 404) ve admin (api/v1/admin/blog.py, /api/v1/admin/blogs: liste, get, POST, PUT, PATCH, DELETE; id + slug). Liste boşken 200 + boş Page. Admin rotaları Faz 5'e kadar korumasız (5.5).</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Faz 4 — Blog (Post) Modülü</t>
+          <t>Faz 4 — Blog Modülü</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1936,7 +1968,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Alembic migration + test_posts.py (draft'ın public listede görünmediğini de test et)</t>
+          <t>Alembic migration + test_blogs.py (yayınlanmamış yazının public listede görünmediğini de test et)</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1960,13 +1992,21 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I32" s="7" t="n"/>
-      <c r="J32" s="4" t="n"/>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: migration uygulandı; tests/test_blogs.py 30 test geçti (admin CRUD, taslağın public'te görünmemesi, sıralama, sayfalama, tag tam eşleşme, reading_time). Toplam 55 test yeşil. Açık not: tag LIKE SQLite'ta büyük/küçük harfe duyarsız, Postgres'te duyarlı.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="25.5" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Faz 4 — Blog (Post) Modülü</t>
+          <t>Faz 4 — Blog Modülü</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -2000,8 +2040,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I33" s="7" t="n"/>
-      <c r="J33" s="4" t="n"/>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Karar verildi: markdown ham dönülüyor (content alanı), frontend render edecek. GET /blogs/{slug} testi içeriğin döndüğünü belgeliyor.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -2040,10 +2088,14 @@
           <t>B-01</t>
         </is>
       </c>
-      <c r="I34" s="7" t="n"/>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Taslak var (models/user.py) ama table=True değil, hashed_password/is_active/is_admin yok.</t>
+          <t>Tamamlandı: models/user.py (tablo users): name (opsiyonel), email (unique+index), hashed_password. Karar: tek kullanıcı olduğu için is_active/is_admin alanları YOK; tablodaki kullanıcı admin sayılır. get_current_admin (5.4) yalnızca 401 dönecek; create_admin.py (5.6) kullanıcı varsa çıkmalı.</t>
         </is>
       </c>
     </row>
@@ -2084,10 +2136,14 @@
           <t>B-01</t>
         </is>
       </c>
-      <c r="I35" s="7" t="n"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>core/security.py şu an boş (0 bayt).</t>
+          <t>Tamamlandı: core/security.py — hash_password/verify_password (pwdlib argon2), create_access_token/decode_access_token (PyJWT HS256; geçersiz/süresi dolmuş token → None). tests/test_security.py 12 test geçti. Not: yayından önce .env'deki JWT_SECRET güçlü (≥32 karakter) bir değerle değiştirilecek.</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2240,7 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Projects ve Posts'un tüm POST/PUT/PATCH/DELETE endpoint'lerini Depends(get_current_admin) ile koru</t>
+          <t>Projects ve Blog'un tüm POST/PUT/PATCH/DELETE endpoint'lerini Depends(get_current_admin) ile koru</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -3296,7 +3352,7 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Faz 4 — Blog (Post) Modülü</t>
+          <t>Faz 4 — Blog Modülü</t>
         </is>
       </c>
       <c r="B10" s="12">

</xml_diff>

<commit_message>
User & Authentication Added & ImageKit connected
</commit_message>
<xml_diff>
--- a/backend/docs/Backend-Proje-Plani-Takip.xlsx
+++ b/backend/docs/Backend-Proje-Plani-Takip.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Görev Takibi" sheetId="1" state="visible" r:id="rId1"/>
@@ -2184,8 +2184,16 @@
           <t>B-01</t>
         </is>
       </c>
-      <c r="I36" s="7" t="n"/>
-      <c r="J36" s="4" t="n"/>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: api/v1/auth.py — POST /api/v1/auth/login (OAuth2PasswordRequestForm, form verisi; yanıt Token: access_token/token_type snake_case, Swagger Authorize uyumlu) ve GET /api/v1/auth/me (UserRead, hashed_password yok). Kullanıcı yoksa da sahte hash'e karşı verify (zamanlama), aynı 401 mesajı + WWW-Authenticate. UserRepository.get_by_email (e-posta küçük harf).</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="25.5" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
@@ -2224,8 +2232,16 @@
           <t>B-01</t>
         </is>
       </c>
-      <c r="I37" s="7" t="n"/>
-      <c r="J37" s="4" t="n"/>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: app/dependencies.py — oauth2_scheme (tokenUrl=/api/v1/auth/login) + get_current_admin: token çöz → e-posta → kullanıcı; geçersiz/süresi dolmuş/kullanıcısı yok → aynı 401. Tek kullanıcı: 403 yok.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="25.5" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -2264,8 +2280,16 @@
           <t>B-01</t>
         </is>
       </c>
-      <c r="I38" s="7" t="n"/>
-      <c r="J38" s="4" t="n"/>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: admin/blogs.py ve admin/projects.py router'larına dependencies=[Depends(get_current_admin)] (18 admin rotası korumalı). Public GET'ler ve /auth/login açık. Testlerde conftest 'client' artık token'lı, 'anon_client' token'sız.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
@@ -2304,8 +2328,16 @@
           <t>B-01</t>
         </is>
       </c>
-      <c r="I39" s="7" t="n"/>
-      <c r="J39" s="4" t="n"/>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: scripts/create_admin.py (python -m scripts.create_admin): e-posta + getpass (min 8, tekrar), kullanıcı yoksa oluşturur, varsa şifre sıfırlar, ikinci kullanıcıyı reddeder. Şifre değiştirme bu script ile (endpoint yok). tests/test_create_admin.py 3 test.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="25.5" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -2344,8 +2376,16 @@
           <t>B-14</t>
         </is>
       </c>
-      <c r="I40" s="7" t="n"/>
-      <c r="J40" s="4" t="n"/>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: tests/test_auth.py (login, me, bozuk/süresi dolmuş/yanlış anahtarlı/kullanıcısı olmayan token, OpenAPI'den taranan 18 admin rotasının tamamı token'sız 401, public rotalar açık) + conftest.py'ye admin_user/client/anon_client fixture'ları. Toplam 131 test yeşil. Not: 5.1 açıklamasındaki is_active/is_admin kararla kaldırıldı.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="25.5" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -2384,10 +2424,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I41" s="7" t="n"/>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Kısmen: imagekitio==5.9.0 pinli. IMAGEKIT_* ayarları Settings'te yok.</t>
+          <t>Tamamlandı: imagekitio==5.9.0 pinli; IMAGEKIT_PUBLIC_KEY / PRIVATE_KEY (SecretStr) / URL_ENDPOINT Settings'te; test conftest'inde sahte değerler.</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2448,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>services/media_service.py: MIME + boyut doğrulama (maks 5MB; jpeg/png/webp), ImageKit upload, url+file_id kaydet</t>
+          <t>services/media_service.py: ImageKit signed-upload parametreleri (token/expire/signature) üret + dosya silme (backend dosya yüklemez, tarayıcı doğrudan ImageKit'e yükler)</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -2428,8 +2472,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I42" s="7" t="n"/>
-      <c r="J42" s="4" t="n"/>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: AsyncImageKit istemcisi, async get_upload_params() (SDK'nın helper'ı coroutine döndürür, await şart) ve delete_file(). Karar: MIME/boyut doğrulaması backend'de değil, ImageKit tarafında (signed upload).</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -2444,7 +2496,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>POST /api/v1/media/upload (admin-only) + DELETE /api/v1/media/{file_id}</t>
+          <t>GET /api/v1/admin/media/auth (UploadAuth: token, expire, signature, publicKey, urlEndpoint) + DELETE /api/v1/admin/media/{file_id} (204; ImageKitError→502)</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -2468,8 +2520,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I43" s="7" t="n"/>
-      <c r="J43" s="4" t="n"/>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı: admin-media router (get_current_admin korumalı), tests/test_media.py (auth şeması, private key sızmaz, token'sız 401, silme 204/502, SDK çıktısı şemaya uyuyor) + conftest'te ağsız sahte delete fixture'ı; admin rota taraması 18→20.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -3533,7 +3593,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -3580,7 +3640,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="25.5" customHeight="1">
+    <row r="2" hidden="1" ht="25.5" customHeight="1">
       <c r="A2" s="21" t="inlineStr">
         <is>
           <t>B-01</t>
@@ -3606,9 +3666,13 @@
           <t>0.6, Faz 5</t>
         </is>
       </c>
-      <c r="F2" s="7" t="n"/>
-    </row>
-    <row r="3" ht="25.5" customHeight="1">
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" hidden="1" ht="25.5" customHeight="1">
       <c r="A3" s="21" t="inlineStr">
         <is>
           <t>B-02</t>
@@ -3640,7 +3704,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1">
+    <row r="4" hidden="1" ht="15.75" customHeight="1">
       <c r="A4" s="21" t="inlineStr">
         <is>
           <t>B-03</t>
@@ -3666,9 +3730,13 @@
           <t>0.1, 0.2</t>
         </is>
       </c>
-      <c r="F4" s="7" t="n"/>
-    </row>
-    <row r="5" ht="25.5" customHeight="1">
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" hidden="1" ht="25.5" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
           <t>B-04</t>
@@ -3726,7 +3794,11 @@
           <t>1.3</t>
         </is>
       </c>
-      <c r="F6" s="7" t="n"/>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="21" t="inlineStr">
@@ -3754,9 +3826,13 @@
           <t>3.1, 3.2</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="25.5" customHeight="1">
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" hidden="1" ht="25.5" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
         <is>
           <t>B-07</t>
@@ -3814,7 +3890,11 @@
           <t>1.8</t>
         </is>
       </c>
-      <c r="F9" s="7" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="21" t="inlineStr">
@@ -3842,9 +3922,13 @@
           <t>1.6</t>
         </is>
       </c>
-      <c r="F10" s="7" t="n"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" hidden="1" ht="15.75" customHeight="1">
       <c r="A11" s="21" t="inlineStr">
         <is>
           <t>B-10</t>
@@ -3876,7 +3960,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1">
+    <row r="12" hidden="1" ht="15.75" customHeight="1">
       <c r="A12" s="21" t="inlineStr">
         <is>
           <t>B-11</t>
@@ -3908,7 +3992,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1">
+    <row r="13" hidden="1" ht="15.75" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
         <is>
           <t>B-12</t>
@@ -3968,7 +4052,7 @@
       </c>
       <c r="F14" s="7" t="n"/>
     </row>
-    <row r="15" ht="15.75" customHeight="1">
+    <row r="15" hidden="1" ht="15.75" customHeight="1">
       <c r="A15" s="21" t="inlineStr">
         <is>
           <t>B-14</t>
@@ -3994,9 +4078,13 @@
           <t>2.1, 2.2, 5.7</t>
         </is>
       </c>
-      <c r="F15" s="7" t="n"/>
-    </row>
-    <row r="16" ht="15.75" customHeight="1">
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" hidden="1" ht="15.75" customHeight="1">
       <c r="A16" s="21" t="inlineStr">
         <is>
           <t>B-15</t>
@@ -4028,7 +4116,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1">
+    <row r="17" hidden="1" ht="15.75" customHeight="1">
       <c r="A17" s="21" t="inlineStr">
         <is>
           <t>B-16</t>
@@ -4060,7 +4148,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1">
+    <row r="18" hidden="1" ht="15.75" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
         <is>
           <t>B-17</t>
@@ -4092,7 +4180,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" hidden="1" ht="15.75" customHeight="1">
       <c r="A19" s="21" t="inlineStr">
         <is>
           <t>B-18</t>
@@ -4124,7 +4212,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
+    <row r="20" hidden="1" ht="15.75" customHeight="1">
       <c r="A20" s="21" t="inlineStr">
         <is>
           <t>B-19</t>
@@ -4156,7 +4244,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="25.5" customHeight="1">
+    <row r="21" hidden="1" ht="25.5" customHeight="1">
       <c r="A21" s="21" t="inlineStr">
         <is>
           <t>B-20</t>
@@ -4214,7 +4302,11 @@
           <t>1.7</t>
         </is>
       </c>
-      <c r="F22" s="7" t="n"/>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="21" t="inlineStr">
@@ -4245,7 +4337,11 @@
       <c r="F23" s="7" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F23"/>
+  <autoFilter ref="A1:F23">
+    <filterColumn colId="5" hiddenButton="0" showButton="1">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="A2:F23">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>$F2="✓"</formula>

</xml_diff>